<commit_message>
implemented most parts of postprocessing between Flim fitting and plotting
</commit_message>
<xml_diff>
--- a/FLIM_fitting/datatoanalyze.xlsx
+++ b/FLIM_fitting/datatoanalyze.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
   <si>
     <t xml:space="preserve">/n/home00/xyang14/Desktop/Metab_Imaging</t>
   </si>
@@ -94,16 +94,16 @@
     <t xml:space="preserve">Comment</t>
   </si>
   <si>
-    <t xml:space="preserve">e20190528_new_scope_o2_drop_40C_1_oxy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/home/mx/Desktop/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190528_new_scope_o2_drop_40C_1_oxy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/home/mx/Desktop/mitoFluxGradients/data/EXP_temperatureResolved/FLIM_fitting_results</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/home/mx/Desktop/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190528_new_scope_o2_drop_40C_1_oxy/irf</t>
+    <t xml:space="preserve">e20190519_new_scope_o2_drop_22C_oxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190519_new_scope_o2_drop_22C_oxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/FLIM_fitting_results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190519_new_scope_o2_drop_22C_oxy/irf</t>
   </si>
   <si>
     <t xml:space="preserve">/Users/photoon/Desktop/metabolic_imaging_20181105/data_analysis/photoon_pc_20181105/systematic_o2_drop/CT/test2/fad.ilp</t>
@@ -115,13 +115,22 @@
     <t xml:space="preserve">AKSOM</t>
   </si>
   <si>
-    <t xml:space="preserve">e20190528_new_scope_o2_drop_40C_2_oxy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/home/mx/Desktop/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190528_new_scope_o2_drop_40C_2_oxy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/home/mx/Desktop/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190528_new_scope_o2_drop_40C_2_oxy/irf</t>
+    <t xml:space="preserve">e20190521_new_scope_o2_drop_22C_oxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190521_new_scope_o2_drop_22C_oxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190521_new_scope_o2_drop_22C_oxy/irf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e20190525_new_scope_o2_drop_22C_oxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190525_new_scope_o2_drop_22C_oxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/mx/mitoFluxGradients/data/EXP_temperatureResolved/raw_sdt_files/e20190525_new_scope_o2_drop_22C_oxy/irf</t>
   </si>
 </sst>
 </file>
@@ -395,7 +404,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43"/>
@@ -577,6 +586,50 @@
         <v>30</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>256</v>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>256</v>
+      </c>
+      <c r="M5" s="1" t="n">
+        <v>280</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>